<commit_message>
Update dependency FrCore dependency to 1.0.1 (#205)
* update FrCore dependency

* prepare release

* update publication request deb256d1bc35418681b9bbc6e16c0622eb0193a0
</commit_message>
<xml_diff>
--- a/ig/CodeSystem-as-cs-intern-id-systems.xlsx
+++ b/ig/CodeSystem-as-cs-intern-id-systems.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0</t>
+    <t>1.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-04-10T13:25:16+00:00</t>
+    <t>2024-04-25T11:50:43+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>